<commit_message>
Add jsw-footer block options
Automated migration updates generated by Experience Modernization Agent.

Changed files: 8
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-jsw-footer.report.xlsx
+++ b/tools/importer/reports/import-jsw-footer.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="67">
   <si>
     <t>_reportFile</t>
   </si>
@@ -124,7 +124,16 @@
     <t>jsw-footer</t>
   </si>
   <si>
-    <t>2026-10-27T16:58:01.393Z</t>
+    <t>2026-10-28T04:42:16.807Z</t>
+  </si>
+  <si>
+    <t>jsw-nav.report.json</t>
+  </si>
+  <si>
+    <t>jsw-nav</t>
+  </si>
+  <si>
+    <t>2026-10-28T04:15:09.687Z</t>
   </si>
   <si>
     <t>jsw-nev-collage.report.json</t>
@@ -175,7 +184,7 @@
     <t>jsw-phase-5.report.json</t>
   </si>
   <si>
-    <t>2026-10-27T08:28:50.476Z</t>
+    <t>2026-10-27T17:17:42.351Z</t>
   </si>
   <si>
     <t>jsw-reserve.report.json</t>
@@ -591,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
@@ -903,8 +912,8 @@
       <c r="D7" t="s">
         <v>16</v>
       </c>
-      <c r="E7">
-        <v>9</v>
+      <c r="E7" t="s">
+        <v>16</v>
       </c>
       <c r="F7" t="s">
         <v>16</v>
@@ -947,11 +956,11 @@
       <c r="C8" t="s">
         <v>16</v>
       </c>
-      <c r="D8" t="b">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>16</v>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8">
+        <v>9</v>
       </c>
       <c r="F8" t="s">
         <v>16</v>
@@ -965,8 +974,8 @@
       <c r="I8" t="s">
         <v>16</v>
       </c>
-      <c r="J8" t="b">
-        <v>0</v>
+      <c r="J8" t="s">
+        <v>16</v>
       </c>
       <c r="K8" t="s">
         <v>18</v>
@@ -978,42 +987,42 @@
         <v>43</v>
       </c>
       <c r="N8" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="O8" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" t="s">
         <v>45</v>
       </c>
-      <c r="B9">
-        <v>5</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" t="s">
-        <v>46</v>
-      </c>
       <c r="H9" t="s">
         <v>16</v>
       </c>
       <c r="I9" t="s">
         <v>16</v>
       </c>
-      <c r="J9" t="s">
-        <v>16</v>
+      <c r="J9" t="b">
+        <v>0</v>
       </c>
       <c r="K9" t="s">
         <v>18</v>
@@ -1022,21 +1031,21 @@
         <v>16</v>
       </c>
       <c r="M9" t="s">
+        <v>46</v>
+      </c>
+      <c r="N9" t="s">
+        <v>30</v>
+      </c>
+      <c r="O9" t="s">
         <v>47</v>
-      </c>
-      <c r="N9" t="s">
-        <v>46</v>
-      </c>
-      <c r="O9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>48</v>
       </c>
-      <c r="B10" t="s">
-        <v>16</v>
+      <c r="B10">
+        <v>5</v>
       </c>
       <c r="C10" t="s">
         <v>16</v>
@@ -1047,14 +1056,14 @@
       <c r="E10" t="s">
         <v>16</v>
       </c>
-      <c r="F10" t="b">
-        <v>1</v>
+      <c r="F10" t="s">
+        <v>16</v>
       </c>
       <c r="G10" t="s">
         <v>49</v>
       </c>
-      <c r="H10">
-        <v>21</v>
+      <c r="H10" t="s">
+        <v>16</v>
       </c>
       <c r="I10" t="s">
         <v>16</v>
@@ -1072,15 +1081,15 @@
         <v>50</v>
       </c>
       <c r="N10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="O10" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
         <v>16</v>
@@ -1094,11 +1103,11 @@
       <c r="E11" t="s">
         <v>16</v>
       </c>
-      <c r="F11" t="s">
-        <v>16</v>
+      <c r="F11" t="b">
+        <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H11">
         <v>21</v>
@@ -1116,18 +1125,18 @@
         <v>16</v>
       </c>
       <c r="M11" t="s">
+        <v>53</v>
+      </c>
+      <c r="N11" t="s">
         <v>54</v>
       </c>
-      <c r="N11" t="s">
-        <v>51</v>
-      </c>
       <c r="O11" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -1145,10 +1154,10 @@
         <v>16</v>
       </c>
       <c r="G12" t="s">
-        <v>56</v>
-      </c>
-      <c r="H12" t="s">
-        <v>16</v>
+        <v>54</v>
+      </c>
+      <c r="H12">
+        <v>21</v>
       </c>
       <c r="I12" t="s">
         <v>16</v>
@@ -1166,7 +1175,7 @@
         <v>57</v>
       </c>
       <c r="N12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="O12" t="s">
         <v>34</v>
@@ -1179,8 +1188,8 @@
       <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="C13">
-        <v>6</v>
+      <c r="C13" t="s">
+        <v>16</v>
       </c>
       <c r="D13" t="s">
         <v>16</v>
@@ -1226,8 +1235,8 @@
       <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="C14" t="s">
-        <v>16</v>
+      <c r="C14">
+        <v>6</v>
       </c>
       <c r="D14" t="s">
         <v>16</v>
@@ -1244,8 +1253,8 @@
       <c r="H14" t="s">
         <v>16</v>
       </c>
-      <c r="I14">
-        <v>5</v>
+      <c r="I14" t="s">
+        <v>16</v>
       </c>
       <c r="J14" t="s">
         <v>16</v>
@@ -1263,6 +1272,53 @@
         <v>62</v>
       </c>
       <c r="O14" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15">
+        <v>5</v>
+      </c>
+      <c r="J15" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15" t="s">
+        <v>18</v>
+      </c>
+      <c r="L15" t="s">
+        <v>16</v>
+      </c>
+      <c r="M15" t="s">
+        <v>66</v>
+      </c>
+      <c r="N15" t="s">
+        <v>65</v>
+      </c>
+      <c r="O15" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>